<commit_message>
Fix VoiceRecorder component filename case
</commit_message>
<xml_diff>
--- a/backend/chat_history.xlsx
+++ b/backend/chat_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1646,6 +1646,134 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>chat_1785298802306</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies today?</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>chat_1785298802306</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>voice_1785298802306</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies today?</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>voice_1785298802306</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add backend config for render
</commit_message>
<xml_diff>
--- a/backend/chat_history.xlsx
+++ b/backend/chat_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1774,6 +1774,904 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>adf</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>chat_1785302099951</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>It seems like you typed a random combination of letters. Could you please rephrase or ask a question so I can assist you better?</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>chat_1785302099951</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>voice_1785302099951</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies today?</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>voice_1785302099951</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> hello</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>voice_1785302099951</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies today?</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>voice_1785302099951</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>chat_1785303484971</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies today?</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>chat_1785303484971</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>who are you</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>chat_1785303484971</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>I am Sylvia AI, an educational assistant for Jesus and Mary Academy students, here to help with your questions and provide information.</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>chat_1785303484971</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>chat_1785303835014</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies today?</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>chat_1785303835014</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>who are you</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>chat_1785303835014</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>I am Sylvia AI, an educational assistant for Jesus and Mary Academy students, here to help with your queries and provide information.</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>chat_1785303835014</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>voice_1785303878285</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies today?</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>voice_1785303878285</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>voice_1785306186266</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies today?</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>voice_1785306186266</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> I like to know about some interesting things about a science letters I am not a Science Students but if I am expecting someone to be a science how a science into St student can reply about it that what is the science</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>voice_1785306186266</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>9801313994</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>If someone asks a science student "What is science?", they might reply:
+"Science is a way of understanding the world around us by observing, experimenting, and drawing conclusions based on evidence. It's like being a detective, trying to figure out how things work and why things happen. Science is all about curiosity, discovery, and learning about the natural world, from the tiny atoms to the vast universe."
+This response shows that the student has a basic understanding of what science is and can explain it in simple terms.</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>voice_1785306186266</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>9999999999</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>chat_1785314683528</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>9999999999</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies today?</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>chat_1785314683528</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>9999999999</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>hello</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>voice_1785314683528</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>9999999999</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies or any questions you have about Jesus and Mary Academy?</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>voice_1785314683528</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>9999999999</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>chat_1785314824286</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>9999999999</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies today?</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>chat_1785314824286</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>9999999999</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>chat_1785314946372</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>9999999999</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Hello. How can I assist you with your studies today?</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>chat_1785314946372</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>chat</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>